<commit_message>
Complete ECOI inventory batches with Penna evidence
Co-authored-by: SherryYoYo6 <SherryYoYo6@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Inventory_batch01.xlsx
+++ b/Inventory_batch01.xlsx
@@ -438,14 +438,14 @@
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
-    <col width="35" customWidth="1" min="18" max="18"/>
+    <col width="40" customWidth="1" min="18" max="18"/>
     <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="35" customWidth="1" min="20" max="20"/>
+    <col width="40" customWidth="1" min="20" max="20"/>
     <col width="55" customWidth="1" min="21" max="21"/>
     <col width="16" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
@@ -469,7 +469,7 @@
     <col width="16" customWidth="1" min="41" max="41"/>
     <col width="16" customWidth="1" min="42" max="42"/>
     <col width="16" customWidth="1" min="43" max="43"/>
-    <col width="90" customWidth="1" min="44" max="44"/>
+    <col width="95" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -746,7 +746,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
+          <t>No high-confidence match</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr"/>
@@ -757,7 +757,7 @@
       <c r="R2" s="2" t="inlineStr"/>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
@@ -802,7 +802,7 @@
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AC2" s="2" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="AR2" s="2" t="inlineStr">
         <is>
-          <t>Official USDA-ARS Riesel/Blacklands page and ARS publication describe long-term precipitation/runoff records, shallow groundwater wells, and public hydrologic database access. Soil-water observations are indicated in the watershed literature, but a specific public soil-moisture download was not verified. No evidence found for isotopes, snow/SWE, or event piezometer/VSA products.</t>
+          <t>Official USDA-ARS Riesel/Blacklands page and ARS publication describe long-term precipitation/runoff records, shallow groundwater wells, and public hydrologic database access. Soil-water observations are indicated in the watershed literature, but a specific public soil-moisture download was not verified. No evidence found for isotopes, snow/SWE, or event piezometer/VSA products. No high-confidence Penna catchment match found in available Part2 fuzzy matching. Official/project source override applied for public-data status.</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
+          <t>No high-confidence match</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -949,7 +949,7 @@
       <c r="R3" s="2" t="inlineStr"/>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>No public download identified</t>
+          <t>N</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="AR3" s="2" t="inlineStr">
         <is>
-          <t>CB1 publications document sprinkling/rain gauges, weirs/discharge, 223 piezometers, 100 tensiometers, 42 TDR pairs, lysimeters, and deuterium/tracer observations. No official public repository or downloadable original dataset was identified; monitoring ended after landslides.</t>
+          <t>CB1 publications document sprinkling/rain gauges, weirs/discharge, 223 piezometers, 100 tensiometers, 42 TDR pairs, lysimeters, and deuterium/tracer observations. No official public repository or downloadable original dataset was identified; monitoring ended after landslides. No high-confidence Penna catchment match found in available Part2 fuzzy matching.</t>
         </is>
       </c>
     </row>
@@ -1130,7 +1130,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
+          <t>No high-confidence match</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr"/>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="AR4" s="2" t="inlineStr">
         <is>
-          <t>OZCAR/AMMA-CATCH sources describe the Upper Oueme/Donga monitoring network with dense rainfall, stream gauges, soil moisture profiles, piezometers/groundwater, geochemical campaigns, isotopes, and EC. Portal-level access is documented, but direct public downloads for the Aguima subcatchment were not verified.</t>
+          <t>OZCAR/AMMA-CATCH sources describe the Upper Oueme/Donga monitoring network with dense rainfall, stream gauges, soil moisture profiles, piezometers/groundwater, geochemical campaigns, isotopes, and EC. Portal-level access is documented, but direct public downloads for the Aguima subcatchment were not verified. No high-confidence Penna catchment match found in available Part2 fuzzy matching.</t>
         </is>
       </c>
     </row>
@@ -1322,23 +1322,43 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="inlineStr"/>
-      <c r="O5" s="2" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shale Hills </t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>49; 100; 159; 160; 216; 240; 241</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>E; E+M; M</t>
+        </is>
+      </c>
       <c r="P5" s="2" t="inlineStr"/>
-      <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>S; S+SS; SS</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>(Perched) WT/GW dynamics and changes in GW storage; Groundwater - streamflow threshold; IEOF; Lateral flow; Macropore flow (no specifical vert/lat); Matrix flow; Pipe flow; Preferential flow (no specifica vert/lat); Return flow/interflow; Soil moisture -groundwater threshold; Soil moisture and rainfall -streamflow threshold; Soil moisture- streamflow threshold; SubFlow; Subsurface hillslope-stream connectivity; Vertical flow; Vertical preferential flow; Water movement through bedrock or at the soil/bedrock interface (either SubFlow or GW rise)</t>
+        </is>
+      </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>CZO Archive / CUAHSI HydroShare</t>
+          <t>CZO Archive / CUAHSI HydroShare Shale Hills</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
@@ -1403,22 +1423,22 @@
       </c>
       <c r="AG5" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AI5" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="AJ5" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AK5" s="2" t="inlineStr">
@@ -1458,7 +1478,7 @@
       </c>
       <c r="AR5" s="2" t="inlineStr">
         <is>
-          <t>CZO Archive and HydroShare list public Shale Hills datasets for precipitation/meteorology, streamflow/discharge, groundwater depth, soil moisture, stable isotopes, groundwater/stream chemistry, EC, and snow depth/reanalysis products. Multi-layer soil moisture and event piezometer network access were not confirmed from the reviewed records.</t>
+          <t>CZO Archive and HydroShare list public Shale Hills datasets for precipitation/meteorology, streamflow/discharge, groundwater depth, soil moisture, stable isotopes, groundwater/stream chemistry, EC, and snow depth/reanalysis products. Multi-layer soil moisture and event piezometer network access were not confirmed from the reviewed records. Penna supporting match: Shale Hills  (Lin et al., 2006a; Lin et al., 2006b; Curtu et al., 2014; Guo et al., 2018; Scaife et al., 2020; Tang et al., 2020); Penna evidence was used only for Observed flags, not public access. Official/project source override applied for public-data status.</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1534,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
+          <t>No high-confidence match</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr"/>
@@ -1525,7 +1545,7 @@
       <c r="R6" s="2" t="inlineStr"/>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T6" s="2" t="inlineStr">
@@ -1550,7 +1570,7 @@
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="Y6" s="2" t="inlineStr">
@@ -1590,7 +1610,7 @@
       </c>
       <c r="AF6" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AG6" s="2" t="inlineStr">
@@ -1650,7 +1670,7 @@
       </c>
       <c r="AR6" s="2" t="inlineStr">
         <is>
-          <t>IML-CZO publications describe an observational network with continuous water/solute fluxes and event-based water-table measurements. HydroShare has public Allerton tile/stage records with EC and Upper Sangamon soil-related resources; a direct precipitation, groundwater, isotope, or snow/SWE download for the Allerton watershed was not verified.</t>
+          <t>IML-CZO publications describe an observational network with continuous water/solute fluxes and event-based water-table measurements. HydroShare has public Allerton tile/stage records with EC and Upper Sangamon soil-related resources; a direct precipitation, groundwater, isotope, or snow/SWE download for the Allerton watershed was not verified. No high-confidence Penna catchment match found in available Part2 fuzzy matching.</t>
         </is>
       </c>
     </row>
@@ -1706,7 +1726,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
+          <t>No high-confidence match</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr"/>
@@ -1717,7 +1737,7 @@
       <c r="R7" s="2" t="inlineStr"/>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>No public download identified</t>
+          <t>N</t>
         </is>
       </c>
       <c r="T7" s="2" t="inlineStr">
@@ -1842,7 +1862,7 @@
       </c>
       <c r="AR7" s="2" t="inlineStr">
         <is>
-          <t>The cited Hydrological Sciences Journal paper analyzes climatic water balance and runoff components in a poorly gauged tropical forested catchment, supporting rainfall and discharge observations. Searches did not locate an official Rompeviento/El Nancite data portal or public downloads; other variables remain uncertain.</t>
+          <t>The cited Hydrological Sciences Journal paper analyzes climatic water balance and runoff components in a poorly gauged tropical forested catchment, supporting rainfall and discharge observations. Searches did not locate an official Rompeviento/El Nancite data portal or public downloads; other variables remain uncertain. No high-confidence Penna catchment match found in available Part2 fuzzy matching.</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1918,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
+          <t>No high-confidence match</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr"/>
@@ -1909,7 +1929,7 @@
       <c r="R8" s="2" t="inlineStr"/>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>No public download identified</t>
+          <t>N</t>
         </is>
       </c>
       <c r="T8" s="2" t="inlineStr">
@@ -2034,7 +2054,7 @@
       </c>
       <c r="AR8" s="2" t="inlineStr">
         <is>
-          <t>Casper et al. report DOC and oxygen-isotope measurements in precipitation, soil water, and runoff to separate flow pathways and infer saturation-excess/contributing areas. No official downloadable Duerreychbachtal repository was identified.</t>
+          <t>Casper et al. report DOC and oxygen-isotope measurements in precipitation, soil water, and runoff to separate flow pathways and infer saturation-excess/contributing areas. No official downloadable Duerreychbachtal repository was identified. No high-confidence Penna catchment match found in available Part2 fuzzy matching.</t>
         </is>
       </c>
     </row>
@@ -2090,7 +2110,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
+          <t>No high-confidence match</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr"/>
@@ -2101,7 +2121,7 @@
       <c r="R9" s="2" t="inlineStr"/>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T9" s="2" t="inlineStr">
@@ -2166,7 +2186,7 @@
       </c>
       <c r="AF9" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="AG9" s="2" t="inlineStr">
@@ -2226,7 +2246,7 @@
       </c>
       <c r="AR9" s="2" t="inlineStr">
         <is>
-          <t>HydroShare Catalina-Jemez CZO has public Marshall Gulch precipitation, streamflow/discharge, and multi-depth soil moisture resources; stream-water chemistry includes stable isotopes and EC. Deep critical-zone/groundwater observations are described in publications, but a groundwater-level public download was not confirmed.</t>
+          <t>HydroShare Catalina-Jemez CZO has public Marshall Gulch precipitation, streamflow/discharge, and multi-depth soil moisture resources; stream-water chemistry includes stable isotopes and EC. Deep critical-zone/groundwater observations are described in publications, but a groundwater-level public download was not confirmed. No high-confidence Penna catchment match found in available Part2 fuzzy matching. Official/project source override applied for public-data status.</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2302,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
+          <t>No high-confidence match</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr"/>
@@ -2308,7 +2328,7 @@
       </c>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="W10" s="2" t="inlineStr">
@@ -2343,12 +2363,12 @@
       </c>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -2418,7 +2438,7 @@
       </c>
       <c r="AR10" s="2" t="inlineStr">
         <is>
-          <t>Official HOAL/BAW sources describe hundreds of sensors for precipitation, runoff at surface/drainage/spring stations, soil moisture, groundwater, water chemistry, and stable-isotope analyses. Search results did not verify an open sensor-data download; access appears via project contact/collaboration or limited site records.</t>
+          <t>Official HOAL/BAW sources describe hundreds of sensors for precipitation, runoff at surface/drainage/spring stations, soil moisture, groundwater, water chemistry, and stable-isotope analyses. Search results did not verify an open sensor-data download; access appears via project contact/collaboration or limited site records. No high-confidence Penna catchment match found in available Part2 fuzzy matching. Official/project source override applied for public-data status.</t>
         </is>
       </c>
     </row>
@@ -2474,7 +2494,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
+          <t>No high-confidence match</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr"/>
@@ -2610,7 +2630,7 @@
       </c>
       <c r="AR11" s="2" t="inlineStr">
         <is>
-          <t>USGS/NRC sources document Yucca Mountain precipitation quantity/chemistry/stable isotopes, surface-water discharge reports, and groundwater levels/water quality. These are official sources, but a single public experimental-watershed download portal was not verified; surface-water access is treated as partial.</t>
+          <t>USGS/NRC sources document Yucca Mountain precipitation quantity/chemistry/stable isotopes, surface-water discharge reports, and groundwater levels/water quality. These are official sources, but a single public experimental-watershed download portal was not verified; surface-water access is treated as partial. No high-confidence Penna catchment match found in available Part2 fuzzy matching.</t>
         </is>
       </c>
     </row>
@@ -2666,7 +2686,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
+          <t>No high-confidence match</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr"/>
@@ -2682,7 +2702,7 @@
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>AgrHyS Observatory / Recherche Data Gouv</t>
+          <t>AgrHyS Observatory / OZCAR / Recherche Data Gouv</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
@@ -2767,12 +2787,12 @@
       </c>
       <c r="AK12" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="AL12" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="AM12" s="2" t="inlineStr">
@@ -2802,7 +2822,7 @@
       </c>
       <c r="AR12" s="2" t="inlineStr">
         <is>
-          <t>Fovet et al. identify Kerrien as an AgrHyS headwater catchment with hourly rainfall, 10-min discharge, 15-min groundwater levels in three piezometers, and 30-min soil moisture at seven depths/two profiles. AgrHyS describes time-series visualization/download services and data portals, but direct public access for all Kerrien series was not verified.</t>
+          <t>Fovet et al. identify Kerrien as an AgrHyS headwater catchment with hourly rainfall, 10-min discharge, 15-min groundwater levels in three piezometers, and 30-min soil moisture at seven depths/two profiles. AgrHyS describes time-series visualization/download services and data portals, but direct public access for all Kerrien series was not verified. No high-confidence Penna catchment match found in available Part2 fuzzy matching. Official/project source override applied for public-data status.</t>
         </is>
       </c>
     </row>
@@ -2858,18 +2878,42 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr"/>
-      <c r="N13" s="2" t="inlineStr"/>
-      <c r="O13" s="2" t="inlineStr"/>
-      <c r="P13" s="2" t="inlineStr"/>
-      <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Maimai M8; Maimai M13; Maimai M14; Maimai M15; Maimai M5; Maimai M6; Maimai M7; Maimai M9</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>169; 170</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>E+M</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>Iso+Ions+EC+Dyes</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>S+SS</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>(Perched) WT/GW dynamics and changes in GW storage; Dynamics of saturated areas; Groundwater - streamflow threshold; Lateral flow; Matrix flow; Pipe flow; Preferential flow (no specifica vert/lat); SEOF; Soil moisture-subsurface flow threshold; SubFlow; Vertical flow; Water movement through bedrock or at the soil/bedrock interface (either SubFlow or GW rise)</t>
+        </is>
+      </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T13" s="2" t="inlineStr">
@@ -2939,22 +2983,22 @@
       </c>
       <c r="AG13" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="AH13" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="AI13" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="AJ13" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="AK13" s="2" t="inlineStr">
@@ -2974,7 +3018,7 @@
       </c>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="AO13" s="2" t="inlineStr">
@@ -2994,7 +3038,7 @@
       </c>
       <c r="AR13" s="2" t="inlineStr">
         <is>
-          <t>HydroShare Maimai database is public and includes rainfall-runoff, PET, stable isotopes, soil-water matric potential, water-table depth from wells/tensiometers, trench flow/tracer data, and geochemical analyses from published studies. Multi-layer volumetric soil moisture and event piezometer networks were not clearly identified.</t>
+          <t>HydroShare Maimai database is public and includes rainfall-runoff, PET, stable isotopes, soil-water matric potential, water-table depth from wells/tensiometers, trench flow/tracer data, and geochemical analyses from published studies. Multi-layer volumetric soil moisture and event piezometer networks were not clearly identified. Penna supporting match: Maimai M8; Maimai M13; Maimai M14; Maimai M15; Maimai M5; Maimai M6; Maimai M7; Maimai M9 (McGlynn et al., 2002; McGlynn et al., 2002; McDonnell etal., 2021); Penna evidence was used only for Observed flags, not public access. Official/project source override applied for public-data status.</t>
         </is>
       </c>
     </row>
@@ -3050,28 +3094,48 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr"/>
-      <c r="N14" s="2" t="inlineStr"/>
-      <c r="O14" s="2" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Coweeta WS10; HJ Andrews Look Out; HJ Andrews Mack; HJ Andrews WS01; HJ Andrews WS02; HJ Andrews WS03; HJ Andrews WS08; HJ Andrews WS09 (+1 more)</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>114; 117; 173; 174; 177; 202; 204; 238; 251; 257</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>E; E+M; M</t>
+        </is>
+      </c>
       <c r="P14" s="2" t="inlineStr"/>
-      <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>S; S+SS; SS</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>(Perched) WT/GW dynamics and changes in GW storage; Dynamics of saturated areas; IEOF; Lateral flow; Lateral preferential flow; Macropore flow (no specifical vert/lat); Preferential flow (no specifica vert/lat); SEOF; Slow/deep SubFlow; SubFlow; Subsurface hillslope-stream connectivity; Water movement through bedrock or at the soil/bedrock interface (either SubFlow or GW rise)</t>
+        </is>
+      </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T14" s="2" t="inlineStr">
         <is>
-          <t>Andrews Forest LTER / EDI Data Portal</t>
+          <t>Andrews Forest LTER / EDI</t>
         </is>
       </c>
       <c r="U14" s="2" t="inlineStr">
         <is>
-          <t>https://andlter.forestry.oregonstate.edu/data/abstract.aspx?dbcode=HF024</t>
+          <t>https://andrewsforest.oregonstate.edu/data</t>
         </is>
       </c>
       <c r="V14" s="2" t="inlineStr">
@@ -3126,27 +3190,27 @@
       </c>
       <c r="AF14" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AG14" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="AH14" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AI14" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="AJ14" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AK14" s="2" t="inlineStr">
@@ -3186,7 +3250,7 @@
       </c>
       <c r="AR14" s="2" t="inlineStr">
         <is>
-          <t>Andrews LTER HF024 and WS10 portal provide downloadable isotope, chemistry, tracer, streamflow, precipitation, and hillslope soil-moisture records; broader HJA datasets include benchmark precipitation, streamflow, soil moisture/temperature, and snow-related/isotope records. Groundwater monitoring for WS10 is publication-supported but direct public well data were not confirmed.</t>
+          <t>Andrews LTER HF024 and WS10 portal provide downloadable isotope, chemistry, tracer, streamflow, precipitation, and hillslope soil-moisture records; broader HJA datasets include benchmark precipitation, streamflow, soil moisture/temperature, and snow-related/isotope records. Groundwater monitoring for WS10 is publication-supported but direct public well data were not confirmed. Penna supporting match: Coweeta WS10; HJ Andrews Look Out; HJ Andrews Mack; HJ Andrews WS01; HJ Andrews WS02; HJ Andrews WS03; HJ Andrews WS08; HJ Andrews WS09 (+1 more) (Hudson et al., 2021; Hwang et al., 2012; Post and Jones, 2001; Post and Jones, 2001; Tague and Brand, 2001; Moore et al,, 2011 ; Qu et al., 2013; Hudson et al., 2021; Voltz et al., 2013; Wemple et al., 2003; Mirus et al., 2011; Mirus and Loague, 2013; Voltz et al., 2013); Penna evidence was used only for Observed flags, not public access. Official/project source override applied for public-data status.</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3306,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
+          <t>No high-confidence match</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr"/>
@@ -3253,7 +3317,7 @@
       <c r="R15" s="2" t="inlineStr"/>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T15" s="2" t="inlineStr">
@@ -3368,7 +3432,7 @@
       </c>
       <c r="AP15" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AQ15" s="2" t="inlineStr">
@@ -3378,7 +3442,7 @@
       </c>
       <c r="AR15" s="2" t="inlineStr">
         <is>
-          <t>OSM and government portals provide downloadable surface-water quality (including stable isotopes/physical parameters), groundwater quality, and regional hydrometric records; Water Survey of Canada and climate agencies provide flow/precipitation records used in studies. Snow/SWE is relevant to cold-region hydrology but a specific public SWE observation product for the oil sands region was not verified.</t>
+          <t>OSM and government portals provide downloadable surface-water quality (including stable isotopes/physical parameters), groundwater quality, and regional hydrometric records; Water Survey of Canada and climate agencies provide flow/precipitation records used in studies. Snow/SWE is relevant to cold-region hydrology but a specific public SWE observation product for the oil sands region was not verified. No high-confidence Penna catchment match found in available Part2 fuzzy matching.</t>
         </is>
       </c>
     </row>
@@ -3434,7 +3498,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
+          <t>No high-confidence match</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr"/>
@@ -3445,7 +3509,7 @@
       <c r="R16" s="2" t="inlineStr"/>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T16" s="2" t="inlineStr">
@@ -3570,7 +3634,7 @@
       </c>
       <c r="AR16" s="2" t="inlineStr">
         <is>
-          <t>HESS relations page links Pedler Creek model input files on GitHub/Zenodo and cites SA Water Data Services station A5030543. WaterConnect/SA reports document groundwater levels/salinity and hydrochemical/isotope work. Public availability is strongest for model inputs, stream station/government groundwater/salinity records; isotope observations appear study/report-based rather than a verified open time-series download.</t>
+          <t>HESS relations page links Pedler Creek model input files on GitHub/Zenodo and cites SA Water Data Services station A5030543. WaterConnect/SA reports document groundwater levels/salinity and hydrochemical/isotope work. Public availability is strongest for model inputs, stream station/government groundwater/salinity records; isotope observations appear study/report-based rather than a verified open time-series download. No high-confidence Penna catchment match found in available Part2 fuzzy matching.</t>
         </is>
       </c>
     </row>
@@ -3626,7 +3690,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
+          <t>No high-confidence match</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr"/>
@@ -3637,7 +3701,7 @@
       <c r="R17" s="2" t="inlineStr"/>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T17" s="2" t="inlineStr">
@@ -3682,7 +3746,7 @@
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AC17" s="2" t="inlineStr">
@@ -3762,7 +3826,7 @@
       </c>
       <c r="AR17" s="2" t="inlineStr">
         <is>
-          <t>FVA describes long-term water/material-cycle monitoring; GFZ public dataset includes rainfall/throughfall, daily creek discharge, groundwater samples and water table, subsurface flow collectors, elemental chemistry, and Mg/Li isotopes. Public soil-moisture download was not verified although water-budget observations are described.</t>
+          <t>FVA describes long-term water/material-cycle monitoring; GFZ public dataset includes rainfall/throughfall, daily creek discharge, groundwater samples and water table, subsurface flow collectors, elemental chemistry, and Mg/Li isotopes. Public soil-moisture download was not verified although water-budget observations are described. No high-confidence Penna catchment match found in available Part2 fuzzy matching.</t>
         </is>
       </c>
     </row>
@@ -3818,7 +3882,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
+          <t>No high-confidence match</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr"/>
@@ -3829,12 +3893,12 @@
       <c r="R18" s="2" t="inlineStr"/>
       <c r="S18" s="2" t="inlineStr">
         <is>
-          <t>No public download identified</t>
+          <t>N</t>
         </is>
       </c>
       <c r="T18" s="2" t="inlineStr">
         <is>
-          <t>Publication record / Scientific Reports and WRR literature</t>
+          <t>Publication record / Mt. Hermon Aquifer studies</t>
         </is>
       </c>
       <c r="U18" s="2" t="inlineStr">
@@ -3944,7 +4008,7 @@
       </c>
       <c r="AP18" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AQ18" s="2" t="inlineStr">
@@ -3954,7 +4018,7 @@
       </c>
       <c r="AR18" s="2" t="inlineStr">
         <is>
-          <t>Publications describe a poorly gauged transboundary karst aquifer with limited spring discharge, groundwater/head, chemistry/solute and isotope information; sources explicitly note lack of shared direct data, precipitation records, and comprehensive monitoring. Snow is hydrologically important for recharge, but a public Mt. Hermon SWE dataset was not identified.</t>
+          <t>Publications describe a poorly gauged transboundary karst aquifer with limited spring discharge, groundwater/head, chemistry/solute and isotope information; sources explicitly note lack of shared direct data, precipitation records, and comprehensive monitoring. Snow is hydrologically important for recharge, but a public Mt. Hermon SWE dataset was not identified. No high-confidence Penna catchment match found in available Part2 fuzzy matching. Official/project source override applied for public-data status.</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4074,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
+          <t>No high-confidence match</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr"/>
@@ -4026,7 +4090,7 @@
       </c>
       <c r="T19" s="2" t="inlineStr">
         <is>
-          <t>Saxon State Flood Center / B2FIND and literature</t>
+          <t>Saxon State Flood Center / Mulde discharge</t>
         </is>
       </c>
       <c r="U19" s="2" t="inlineStr">
@@ -4046,7 +4110,7 @@
       </c>
       <c r="X19" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="Y19" s="2" t="inlineStr">
@@ -4066,7 +4130,7 @@
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AC19" s="2" t="inlineStr">
@@ -4086,7 +4150,7 @@
       </c>
       <c r="AF19" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AG19" s="2" t="inlineStr">
@@ -4136,7 +4200,7 @@
       </c>
       <c r="AP19" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AQ19" s="2" t="inlineStr">
@@ -4146,7 +4210,7 @@
       </c>
       <c r="AR19" s="2" t="inlineStr">
         <is>
-          <t>Saxon Flood Center provides official downloadable annual discharge lists for Freiberger Mulde gauges. Literature and regional B2FIND/FRED records indicate rain-runoff, soil moisture/piezometer-style hillslope studies, EC, and stable-isotope sampling in Mulde/eastern German systems, but direct public downloads for the cited headwater study variables were not verified.</t>
+          <t>Saxon Flood Center provides official downloadable annual discharge lists for Freiberger Mulde gauges. Literature and regional B2FIND/FRED records indicate rain-runoff, soil moisture/piezometer-style hillslope studies, EC, and stable-isotope sampling in Mulde/eastern German systems, but direct public downloads for the cited headwater study variables were not verified. No high-confidence Penna catchment match found in available Part2 fuzzy matching. Official/project source override applied for public-data status.</t>
         </is>
       </c>
     </row>
@@ -4202,7 +4266,7 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
+          <t>No high-confidence match</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr"/>
@@ -4213,7 +4277,7 @@
       <c r="R20" s="2" t="inlineStr"/>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t>No public download identified</t>
+          <t>N</t>
         </is>
       </c>
       <c r="T20" s="2" t="inlineStr">
@@ -4238,7 +4302,7 @@
       </c>
       <c r="X20" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="Y20" s="2" t="inlineStr">
@@ -4248,7 +4312,7 @@
       </c>
       <c r="Z20" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AA20" s="2" t="inlineStr">
@@ -4328,7 +4392,7 @@
       </c>
       <c r="AP20" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AQ20" s="2" t="inlineStr">
@@ -4338,7 +4402,7 @@
       </c>
       <c r="AR20" s="2" t="inlineStr">
         <is>
-          <t>Regional hydrometeorological service documents meteorological and hydrological posts in Kostroma Oblast, and the cited Upper Volga spring-flood modeling paper implies precipitation/runoff/snowmelt observations. No experimental watershed portal or downloadable observation dataset specific to Kostroma Catchment was identified.</t>
+          <t>Regional hydrometeorological service documents meteorological and hydrological posts in Kostroma Oblast, and the cited Upper Volga spring-flood modeling paper implies precipitation/runoff/snowmelt observations. No experimental watershed portal or downloadable observation dataset specific to Kostroma Catchment was identified. No high-confidence Penna catchment match found in available Part2 fuzzy matching.</t>
         </is>
       </c>
     </row>
@@ -4394,7 +4458,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>Not evaluated - Penna files unavailable in repository</t>
+          <t>No high-confidence match</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr"/>
@@ -4405,7 +4469,7 @@
       <c r="R21" s="2" t="inlineStr"/>
       <c r="S21" s="2" t="inlineStr">
         <is>
-          <t>No public download identified</t>
+          <t>N</t>
         </is>
       </c>
       <c r="T21" s="2" t="inlineStr">
@@ -4530,7 +4594,7 @@
       </c>
       <c r="AR21" s="2" t="inlineStr">
         <is>
-          <t>Point Peter Brook publications document rainfall/throughfall, streamflow/storm runoff, groundwater/riparian and hillslope waters, wetland/riparian source areas, sulfate/chemistry, stable isotope approaches, and snowmelt-season sampling. Searches did not identify a public managed repository for the original watershed observations.</t>
+          <t>Point Peter Brook publications document rainfall/throughfall, streamflow/storm runoff, groundwater/riparian and hillslope waters, wetland/riparian source areas, sulfate/chemistry, stable isotope approaches, and snowmelt-season sampling. Searches did not identify a public managed repository for the original watershed observations. No high-confidence Penna catchment match found in available Part2 fuzzy matching.</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -4554,7 +4618,7 @@
     <col width="55" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="35" customWidth="1" min="6" max="6"/>
-    <col width="90" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4617,7 +4681,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -4627,125 +4691,125 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>CB1, Coos Bay, Oregon, United States</t>
+          <t>Blacklands Experimental Watershed, USDA-ARS Grassland, Soil and Water Research Laboratory watershed, Riesel, Texas, United States</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>McMillan</t>
+          <t>Official_Repository</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>ProcessDatabase3-filtered.xlsx</t>
+          <t>USDA-ARS STEWARDS / Riesel Watershed</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1029/97wr02595</t>
+          <t>https://www.nrrig.mwa.ars.usda.gov/STEWARDS_HTML/Riesel%20Watershed%20TX.htm</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+          <t>Observation/public-data decision support</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>Official Riesel page describes long-term precipitation/runoff, hydrologic data collection, and shallow groundwater monitoring.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Aguima catchment, Upper Oueme, Benin</t>
+          <t>Blacklands Experimental Watershed, USDA-ARS Grassland, Soil and Water Research Laboratory watershed, Riesel, Texas, United States</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>McMillan</t>
+          <t>Official_Repository</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>ProcessDatabase3-filtered.xlsx</t>
+          <t>USDA-ARS publication summary</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.pce.2005.06.005</t>
+          <t>https://www.ars.usda.gov/research/publications/publication/?seqNo115=301178</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+          <t>Observation/public-data decision support</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>ARS summary states legacy discharge, sediment, meteorological, precipitation/baseflow water-quality data are available on the web.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Susquehanna Shale Hills CZO - Shale Hills, United States</t>
+          <t>Blacklands Experimental Watershed, USDA-ARS Grassland, Soil and Water Research Laboratory watershed, Riesel, Texas, United States</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>McMillan</t>
+          <t>Official_Repository</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>ProcessDatabase3-filtered.xlsx</t>
+          <t>USDA-ARS STEWARDS / Riesel Watershed</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.2136/vzj2018.04.0092</t>
+          <t>https://www.nrrig.mwa.ars.usda.gov/STEWARDS_HTML/Riesel%20Watershed%20TX.htm</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+          <t>Official/project repository public-data status and variable availability</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>Official USDA-ARS Riesel/Blacklands page documents public hydrologic data including precipitation, runoff and groundwater-related monitoring.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>IML CZO, Upper Sangamon River Basin, Allerton Trust Farm, United States</t>
+          <t>CB1, Coos Bay, Oregon, United States</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -4760,12 +4824,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1029/2021WR030507</t>
+          <t>https://doi.org/10.1029/97wr02595</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -4775,88 +4839,88 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Rompeviento and El Nancite, Nicaragua, Nicaragua</t>
+          <t>CB1, Coos Bay, Oregon, United States</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>McMillan</t>
+          <t>Publication</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>ProcessDatabase3-filtered.xlsx</t>
+          <t>CB1 hydrologic-response publication PDF</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1080/02626667.2014.964244</t>
+          <t>https://ajsonline.org/article/61638-near-surface-hydrologic-response-for-a-steep-unchanneled-catchment-near-coos-bay-oregon-2-physics-based-simulations.pdf</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+          <t>Observation/public-data decision support</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>Publication documents extensive rain gauges, weirs, piezometers, tensiometers, TDR, lysimeters, and deuterium observations but no public data repository.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Duerreychbachtal, Germany</t>
+          <t>CB1, Coos Bay, Oregon, United States</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>McMillan</t>
+          <t>Publication</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>ProcessDatabase3-filtered.xlsx</t>
+          <t>CB1 site literature DOI</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/S1474-7065(03)00037-8</t>
+          <t>https://doi.org/10.1029/97WR02595</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+          <t>Observation/public-data decision support</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>Original cited paper confirms subsurface-flow-path investigation at CB1.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Marshall Gulch, Santa Catalina Mountains CZO, United States</t>
+          <t>Aguima catchment, Upper Oueme, Benin</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -4871,12 +4935,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1002/hyp.13363</t>
+          <t>https://doi.org/10.1016/j.pce.2005.06.005</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -4886,88 +4950,88 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>HOAL Petzenkirchen, Vienna, Austria</t>
+          <t>Aguima catchment, Upper Oueme, Benin</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>McMillan</t>
+          <t>Project_Website</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>ProcessDatabase3-filtered.xlsx</t>
+          <t>OZCAR/DEIMS AMMA-CATCH Upper Oueme</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.scitotenv.2015.10.151</t>
+          <t>https://deims.org/db22a81e-e7f9-4492-a99e-4a9e0170c4a1</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+          <t>Observation/public-data decision support</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>Official site identifies Upper Oueme as AMMA-CATCH observation network with water-cycle studies.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Yucca Mountain, Nevada, United States</t>
+          <t>Aguima catchment, Upper Oueme, Benin</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>McMillan</t>
+          <t>Project_Website</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>ProcessDatabase3-filtered.xlsx</t>
+          <t>AMMA-CATCH observatory paper PDF</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/S0022-1694(01)00358-4</t>
+          <t>https://ird.hal.science/ird-02153117v1/file/galle%20et%20al%202018.pdf</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+          <t>Observation/public-data decision support</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>Paper describes dense rain gauges, stream gauges, piezometers, soil moisture profiles, isotopes, and EC/geochemical work.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Kerrien catchment, Brittany, France</t>
+          <t>Susquehanna Shale Hills CZO - Shale Hills, United States</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -4982,12 +5046,12 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.5194/hess-19-105-2015</t>
+          <t>https://doi.org/10.2136/vzj2018.04.0092</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -4997,236 +5061,236 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Maimai M8 experimental catchment, New Zealand</t>
+          <t>Susquehanna Shale Hills CZO - Shale Hills, United States</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>McMillan</t>
+          <t>Penna_Part2</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>ProcessDatabase3-filtered.xlsx</t>
+          <t>Penna_globalsynthesis_DB_Part2_update_2026_01.csv</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.jhydrol.2012.05.023</t>
+          <t>https://doi.org/10.5281/zenodo.15123553</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+          <t>Catchment fuzzy match and runoff-process labels</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>Matched to Shale Hills  with process labels: (Perched) WT/GW dynamics and changes in GW storage; Groundwater - streamflow threshold; IEOF; Lateral flow; Macropore flow (no specifical vert/lat); Matrix flow; Pipe flow; Preferential flow (no specifica vert/lat); Return flow/interflow; Soil moisture -groundwater threshold; Soil moisture and rainf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>WS10, H.J. Andrews, Oregon, United States</t>
+          <t>Susquehanna Shale Hills CZO - Shale Hills, United States</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>McMillan</t>
+          <t>Penna_Part1</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>ProcessDatabase3-filtered.xlsx</t>
+          <t>Penna_globalsynthesis_DB_Part1.csv</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.jhydrol.2012.05.023</t>
+          <t>https://doi.org/10.5281/zenodo.15123553</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+          <t>Reference-level approach/tracer/flow type</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>Reference IDs 49; 100; 159; 160; 216; 240; 241; approach=E; E+M; M; tracer=; flow=S; S+SS; SS</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Athabasca Oil Sands region, Alberta, Canada</t>
+          <t>Susquehanna Shale Hills CZO - Shale Hills, United States</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>McMillan</t>
+          <t>Official_Repository</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>ProcessDatabase3-filtered.xlsx</t>
+          <t>Shale Hills CZO Archive datasets</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.ejrh.2015.12.062</t>
+          <t>https://czo-archive.criticalzone.org/shale-hills/data/datasets/</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+          <t>Observation/public-data decision support</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>CZO Archive lists precipitation, soil moisture, groundwater, streamflow, chemistry, stable isotope, and EC datasets.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Pedler Creek, Willunga Basin, Australia</t>
+          <t>Susquehanna Shale Hills CZO - Shale Hills, United States</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>McMillan</t>
+          <t>Official_Repository</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>ProcessDatabase3-filtered.xlsx</t>
+          <t>Shale Hills HydroShare precipitation</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.5194/hess-25-4299-2021</t>
+          <t>http://www.hydroshare.org/resource/417c018edd324a75828195625adbc19f</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+          <t>Observation/public-data decision support</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>HydroShare precipitation/meteorology record includes downloadable precipitation and snow-depth variables.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Conventwald Basin, Black Forest Mountains, Germany</t>
+          <t>Susquehanna Shale Hills CZO - Shale Hills, United States</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>McMillan</t>
+          <t>Official_Repository</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>ProcessDatabase3-filtered.xlsx</t>
+          <t>Shale Hills HydroShare groundwater/discharge</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1002/hyp.142</t>
+          <t>https://www.hydroshare.org/resource/60923e1f1a3d44e39a16260d980db974/</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+          <t>Observation/public-data decision support</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>HydroShare record documents groundwater depth and streamflow/discharge variables.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Mt. Hermon Range, Israel, Syria, and Lebanon</t>
+          <t>Susquehanna Shale Hills CZO - Shale Hills, United States</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>McMillan</t>
+          <t>Official_Repository</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>ProcessDatabase3-filtered.xlsx</t>
+          <t>CZO Archive / CUAHSI HydroShare Shale Hills</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1002/wrcr.20229</t>
+          <t>https://czo-archive.criticalzone.org/shale-hills/data/datasets/</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+          <t>Official/project repository public-data status and variable availability</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>CZO/HydroShare provides public Shale Hills hydrologic, chemistry, isotope, soil moisture, groundwater and snow-related datasets.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Freiberger Mulde, Germany</t>
+          <t>IML CZO, Upper Sangamon River Basin, Allerton Trust Farm, United States</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -5241,12 +5305,12 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s12665-016-5750-y</t>
+          <t>https://doi.org/10.1029/2021WR030507</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -5256,140 +5320,140 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Kostroma Catchment, Russia</t>
+          <t>IML CZO, Upper Sangamon River Basin, Allerton Trust Farm, United States</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>McMillan</t>
+          <t>Official_Repository</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>ProcessDatabase3-filtered.xlsx</t>
+          <t>IML-CZO HydroShare Allerton tiles</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.5194/adgeo-9-115-2006</t>
+          <t>https://www.hydroshare.org/resource/352f073bb68449b1bae259900a0058f3/</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+          <t>Observation/public-data decision support</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>HydroShare Allerton dataset contains hydropedologic properties, stage/depth, and EC for tile-drain monitoring.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Point Peter Brook watershed, New York, United States</t>
+          <t>IML CZO, Upper Sangamon River Basin, Allerton Trust Farm, United States</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>McMillan</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>ProcessDatabase3-filtered.xlsx</t>
+          <t>IML-CZO overview</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.jhydrol.2007.05.007</t>
+          <t>https://ssa.ncsa.illinois.edu/isda/projects/iml-czo/</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+          <t>Observation/public-data decision support</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Primary McMillan-derived row used for watershed name, coordinates, area, citation, and Level-1 runoff process flags.</t>
+          <t>Project page describes Upper Sangamon/Allerton observation network and water, nutrient, sediment flux goals.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Blacklands Experimental Watershed, USDA-ARS Grassland, Soil and Water Research Laboratory watershed, Riesel, Texas, United States</t>
+          <t>Rompeviento and El Nancite, Nicaragua, Nicaragua</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Official_Repository</t>
+          <t>McMillan</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>USDA-ARS STEWARDS / Riesel Watershed</t>
+          <t>ProcessDatabase3-filtered.xlsx</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://www.nrrig.mwa.ars.usda.gov/STEWARDS_HTML/Riesel%20Watershed%20TX.htm</t>
+          <t>https://doi.org/10.1080/02626667.2014.964244</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Watershed metadata and Level-1 runoff process aggregation</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Official Riesel page describes long-term precipitation/runoff, hydrologic data collection, and shallow groundwater monitoring.</t>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Blacklands Experimental Watershed, USDA-ARS Grassland, Soil and Water Research Laboratory watershed, Riesel, Texas, United States</t>
+          <t>Rompeviento and El Nancite, Nicaragua, Nicaragua</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Official_Repository</t>
+          <t>Publication</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>USDA-ARS publication summary</t>
+          <t>Calderon and Uhlenbrook DOI</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://www.ars.usda.gov/research/publications/publication/?seqNo115=301178</t>
+          <t>https://doi.org/10.1080/02626667.2014.964244</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -5404,51 +5468,51 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>ARS summary states legacy discharge, sediment, meteorological, precipitation/baseflow water-quality data are available on the web.</t>
+          <t>Cited paper supports rainfall-runoff/water-balance observations for the Nicaragua catchment; no repository found.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>CB1, Coos Bay, Oregon, United States</t>
+          <t>Duerreychbachtal, Germany</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Publication</t>
+          <t>McMillan</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>CB1 hydrologic-response publication PDF</t>
+          <t>ProcessDatabase3-filtered.xlsx</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://ajsonline.org/article/61638-near-surface-hydrologic-response-for-a-steep-unchanneled-catchment-near-coos-bay-oregon-2-physics-based-simulations.pdf</t>
+          <t>https://doi.org/10.1016/S1474-7065(03)00037-8</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Watershed metadata and Level-1 runoff process aggregation</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Publication documents extensive rain gauges, weirs, piezometers, tensiometers, TDR, lysimeters, and deuterium observations but no public data repository.</t>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>CB1, Coos Bay, Oregon, United States</t>
+          <t>Duerreychbachtal, Germany</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -5458,12 +5522,12 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>CB1 site literature DOI</t>
+          <t>Duerreychbachtal publication DOI</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1029/97WR02595</t>
+          <t>https://doi.org/10.1016/S1474-7065(03)00037-8</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -5478,66 +5542,66 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Original cited paper confirms subsurface-flow-path investigation at CB1.</t>
+          <t>Publication abstract documents DOC and oxygen-isotope observations in precipitation, soil water, and runoff for flow-path separation.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Aguima catchment, Upper Oueme, Benin</t>
+          <t>Marshall Gulch, Santa Catalina Mountains CZO, United States</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Project_Website</t>
+          <t>McMillan</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>OZCAR/DEIMS AMMA-CATCH Upper Oueme</t>
+          <t>ProcessDatabase3-filtered.xlsx</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://deims.org/db22a81e-e7f9-4492-a99e-4a9e0170c4a1</t>
+          <t>https://doi.org/10.1002/hyp.13363</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Watershed metadata and Level-1 runoff process aggregation</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Official site identifies Upper Oueme as AMMA-CATCH observation network with water-cycle studies.</t>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Aguima catchment, Upper Oueme, Benin</t>
+          <t>Marshall Gulch, Santa Catalina Mountains CZO, United States</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Project_Website</t>
+          <t>Official_Repository</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>AMMA-CATCH observatory paper PDF</t>
+          <t>Catalina-Jemez CZO HydroShare group</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://ird.hal.science/ird-02153117v1/file/galle%20et%20al%202018.pdf</t>
+          <t>https://www.hydroshare.org/group/142</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -5552,14 +5616,14 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Paper describes dense rain gauges, stream gauges, piezometers, soil moisture profiles, isotopes, and EC/geochemical work.</t>
+          <t>Group page lists public Marshall Gulch precipitation, soil moisture, streamflow, and chemistry resources.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Susquehanna Shale Hills CZO - Shale Hills, United States</t>
+          <t>Marshall Gulch, Santa Catalina Mountains CZO, United States</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -5569,12 +5633,12 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Shale Hills CZO Archive datasets</t>
+          <t>Marshall Gulch streamflow HydroShare</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://czo-archive.criticalzone.org/shale-hills/data/datasets/</t>
+          <t>https://www.hydroshare.org/resource/3c1fd54381764e5b8865609cb4127d63/</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -5589,14 +5653,14 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>CZO Archive lists precipitation, soil moisture, groundwater, streamflow, chemistry, stable isotope, and EC datasets.</t>
+          <t>HydroShare resource documents 30-minute streamflow/discharge at Marshall Gulch.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Susquehanna Shale Hills CZO - Shale Hills, United States</t>
+          <t>Marshall Gulch, Santa Catalina Mountains CZO, United States</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -5606,12 +5670,12 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Shale Hills HydroShare precipitation</t>
+          <t>Marshall Gulch soil moisture HydroShare</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>http://www.hydroshare.org/resource/417c018edd324a75828195625adbc19f</t>
+          <t>https://www.hydroshare.org/resource/1efcd98af1544905adcb80c79e779c3d/</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -5626,14 +5690,14 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>HydroShare precipitation/meteorology record includes downloadable precipitation and snow-depth variables.</t>
+          <t>HydroShare resource documents soil moisture at various depths in 11 pits.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Susquehanna Shale Hills CZO - Shale Hills, United States</t>
+          <t>Marshall Gulch, Santa Catalina Mountains CZO, United States</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -5643,12 +5707,12 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Shale Hills HydroShare groundwater/discharge</t>
+          <t>Santa Catalina stream chemistry HydroShare</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.hydroshare.org/resource/60923e1f1a3d44e39a16260d980db974/</t>
+          <t>https://www.hydroshare.org/resource/3df05937abfc4cb59b8be04d674c4b48/</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -5663,14 +5727,14 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>HydroShare record documents groundwater depth and streamflow/discharge variables.</t>
+          <t>HydroShare resource documents stream chemistry, EC, and stable isotopes including Marshall Gulch locations.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>IML CZO, Upper Sangamon River Basin, Allerton Trust Farm, United States</t>
+          <t>Marshall Gulch, Santa Catalina Mountains CZO, United States</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -5680,86 +5744,86 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>IML-CZO HydroShare Allerton tiles</t>
+          <t>CUAHSI HydroShare Catalina-Jemez CZO</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.hydroshare.org/resource/352f073bb68449b1bae259900a0058f3/</t>
+          <t>https://www.hydroshare.org/group/142</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Official/project repository public-data status and variable availability</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>HydroShare Allerton dataset contains hydropedologic properties, stage/depth, and EC for tile-drain monitoring.</t>
+          <t>Catalina-Jemez CZO HydroShare provides public Marshall Gulch precipitation, streamflow, soil moisture, groundwater/chemistry and isotope-related resources.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>IML CZO, Upper Sangamon River Basin, Allerton Trust Farm, United States</t>
+          <t>HOAL Petzenkirchen, Vienna, Austria</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>McMillan</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>IML-CZO overview</t>
+          <t>ProcessDatabase3-filtered.xlsx</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://ssa.ncsa.illinois.edu/isda/projects/iml-czo/</t>
+          <t>https://doi.org/10.1016/j.scitotenv.2015.10.151</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Watershed metadata and Level-1 runoff process aggregation</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Project page describes Upper Sangamon/Allerton observation network and water, nutrient, sediment flux goals.</t>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Rompeviento and El Nancite, Nicaragua, Nicaragua</t>
+          <t>HOAL Petzenkirchen, Vienna, Austria</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Publication</t>
+          <t>Project_Website</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Calderon and Uhlenbrook DOI</t>
+          <t>BAW HOAL official page</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1080/02626667.2014.964244</t>
+          <t>https://www.baw.at/en/water-and-soil/research-facilities/hoal.html</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -5774,29 +5838,29 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Cited paper supports rainfall-runoff/water-balance observations for the Nicaragua catchment; no repository found.</t>
+          <t>Official page describes precipitation, runoff, soil moisture, groundwater, water chemistry, and stable isotope monitoring.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Duerreychbachtal, Germany</t>
+          <t>HOAL Petzenkirchen, Vienna, Austria</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Publication</t>
+          <t>Project_Website</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Duerreychbachtal publication DOI</t>
+          <t>HOAL project page</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/S1474-7065(03)00037-8</t>
+          <t>https://hoal.hydrology.at/the-hoal</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -5811,14 +5875,14 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Publication abstract documents DOC and oxygen-isotope observations in precipitation, soil water, and runoff for flow-path separation.</t>
+          <t>Project page describes HOAL as an instrumented catchment with runoff processes, springs, tile drains, and sensors.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Marshall Gulch, Santa Catalina Mountains CZO, United States</t>
+          <t>HOAL Petzenkirchen, Vienna, Austria</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -5828,71 +5892,71 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Catalina-Jemez CZO HydroShare group</t>
+          <t>HOAL Petzenkirchen / BAW-TU Wien</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.hydroshare.org/group/142</t>
+          <t>https://www.baw.at/en/water-and-soil/research-facilities/hoal.html</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Official/project repository public-data status and variable availability</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Group page lists public Marshall Gulch precipitation, soil moisture, streamflow, and chemistry resources.</t>
+          <t>HOAL official sources describe high-density monitoring of precipitation, runoff, soil moisture, groundwater, chemistry and isotopes; access is partly portal/request/collaboration-mediated.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Marshall Gulch, Santa Catalina Mountains CZO, United States</t>
+          <t>Yucca Mountain, Nevada, United States</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Official_Repository</t>
+          <t>McMillan</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Marshall Gulch streamflow HydroShare</t>
+          <t>ProcessDatabase3-filtered.xlsx</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.hydroshare.org/resource/3c1fd54381764e5b8865609cb4127d63/</t>
+          <t>https://doi.org/10.1016/S0022-1694(01)00358-4</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Watershed metadata and Level-1 runoff process aggregation</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>HydroShare resource documents 30-minute streamflow/discharge at Marshall Gulch.</t>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Marshall Gulch, Santa Catalina Mountains CZO, United States</t>
+          <t>Yucca Mountain, Nevada, United States</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -5902,12 +5966,12 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Marshall Gulch soil moisture HydroShare</t>
+          <t>USGS Yucca Mountain precipitation chemistry/isotopes</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.hydroshare.org/resource/1efcd98af1544905adcb80c79e779c3d/</t>
+          <t>https://pubs.usgs.gov/sir/2011/5140/</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -5922,14 +5986,14 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>HydroShare resource documents soil moisture at various depths in 11 pits.</t>
+          <t>USGS report documents event precipitation chemistry and stable isotope observations at Yucca Mountain.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Marshall Gulch, Santa Catalina Mountains CZO, United States</t>
+          <t>Yucca Mountain, Nevada, United States</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -5939,12 +6003,12 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Santa Catalina stream chemistry HydroShare</t>
+          <t>USGS Nevada data portal</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.hydroshare.org/resource/3df05937abfc4cb59b8be04d674c4b48/</t>
+          <t>https://www.usgs.gov/centers/nevada-water-science-center/data</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -5959,51 +6023,51 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>HydroShare resource documents stream chemistry, EC, and stable isotopes including Marshall Gulch locations.</t>
+          <t>USGS Nevada page provides access to public streamflow, groundwater, precipitation, and water-quality data through official systems.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>HOAL Petzenkirchen, Vienna, Austria</t>
+          <t>Kerrien catchment, Brittany, France</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Project_Website</t>
+          <t>McMillan</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>BAW HOAL official page</t>
+          <t>ProcessDatabase3-filtered.xlsx</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.baw.at/en/water-and-soil/research-facilities/hoal.html</t>
+          <t>https://doi.org/10.5194/hess-19-105-2015</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Watershed metadata and Level-1 runoff process aggregation</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Official page describes precipitation, runoff, soil moisture, groundwater, water chemistry, and stable isotope monitoring.</t>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>HOAL Petzenkirchen, Vienna, Austria</t>
+          <t>Kerrien catchment, Brittany, France</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -6013,12 +6077,12 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>HOAL project page</t>
+          <t>AgrHyS monitoring page</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://hoal.hydrology.at/the-hoal</t>
+          <t>https://eng-agrhys.rennes.hub.inrae.fr/monitoring</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -6033,29 +6097,29 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Project page describes HOAL as an instrumented catchment with runoff processes, springs, tile drains, and sensors.</t>
+          <t>AgrHyS page documents monitoring tables and data access/visualization services.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Yucca Mountain, Nevada, United States</t>
+          <t>Kerrien catchment, Brittany, France</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Official_Repository</t>
+          <t>Publication</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>USGS Yucca Mountain precipitation chemistry/isotopes</t>
+          <t>Fovet et al. Kerrien paper PDF</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://pubs.usgs.gov/sir/2011/5140/</t>
+          <t>https://hal.science/hal-01461076v1/file/2015_Fovet_Hydrology%20and%20Earth%20System%20Sciences_1.pdf</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -6070,14 +6134,14 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>USGS report documents event precipitation chemistry and stable isotope observations at Yucca Mountain.</t>
+          <t>Paper explicitly describes Kerrien rainfall, discharge, piezometers, and multi-depth soil moisture observations.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Yucca Mountain, Nevada, United States</t>
+          <t>Kerrien catchment, Brittany, France</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -6087,12 +6151,12 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>USGS Nevada data portal</t>
+          <t>AgrHyS Recherche Data Gouv</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.usgs.gov/centers/nevada-water-science-center/data</t>
+          <t>https://entrepot.recherche.data.gouv.fr/dataverse.xhtml?alias=agrhys</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -6107,7 +6171,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>USGS Nevada page provides access to public streamflow, groundwater, precipitation, and water-quality data through official systems.</t>
+          <t>Dataverse lists AgrHyS/Kervidy public chemistry and high-frequency event datasets.</t>
         </is>
       </c>
     </row>
@@ -6119,12 +6183,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Project_Website</t>
+          <t>Official_Repository</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>AgrHyS monitoring page</t>
+          <t>AgrHyS Observatory / OZCAR / Recherche Data Gouv</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -6134,91 +6198,91 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Official/project repository public-data status and variable availability</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>AgrHyS page documents monitoring tables and data access/visualization services.</t>
+          <t>AgrHyS monitoring pages and data portals document rainfall, discharge, soil moisture, piezometers/groundwater, chemistry, EC and isotope observations; some access is portal/request-mediated.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Kerrien catchment, Brittany, France</t>
+          <t>Maimai M8 experimental catchment, New Zealand</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Publication</t>
+          <t>McMillan</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Fovet et al. Kerrien paper PDF</t>
+          <t>ProcessDatabase3-filtered.xlsx</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://hal.science/hal-01461076v1/file/2015_Fovet_Hydrology%20and%20Earth%20System%20Sciences_1.pdf</t>
+          <t>https://doi.org/10.1016/j.jhydrol.2012.05.023</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Watershed metadata and Level-1 runoff process aggregation</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Paper explicitly describes Kerrien rainfall, discharge, piezometers, and multi-depth soil moisture observations.</t>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Kerrien catchment, Brittany, France</t>
+          <t>Maimai M8 experimental catchment, New Zealand</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Official_Repository</t>
+          <t>Penna_Part2</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>AgrHyS Recherche Data Gouv</t>
+          <t>Penna_globalsynthesis_DB_Part2_update_2026_01.csv</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://entrepot.recherche.data.gouv.fr/dataverse.xhtml?alias=agrhys</t>
+          <t>https://doi.org/10.5281/zenodo.15123553</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Catchment fuzzy match and runoff-process labels</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Dataverse lists AgrHyS/Kervidy public chemistry and high-frequency event datasets.</t>
+          <t xml:space="preserve">Matched to Maimai M8; Maimai M13; Maimai M14; Maimai M15; Maimai M5; Maimai M6; Maimai M7; Maimai M9 with process labels: (Perched) WT/GW dynamics and changes in GW storage; Dynamics of saturated areas; Groundwater - streamflow threshold; Lateral flow; Matrix flow; Pipe flow; Preferential flow (no specifica vert/lat); SEOF; Soil moisture-subsurface flow threshold; SubFlow; Vertical flow; Water movement through bedrock </t>
         </is>
       </c>
     </row>
@@ -6230,32 +6294,32 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Official_Repository</t>
+          <t>Penna_Part1</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Maimai HydroShare repository</t>
+          <t>Penna_globalsynthesis_DB_Part1.csv</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.hydroshare.org/resource/a292cb65a5d24a31a60978b2ab390266/</t>
+          <t>https://doi.org/10.5281/zenodo.15123553</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Reference-level approach/tracer/flow type</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>HydroShare repository contains public Maimai M8 rainfall-runoff, isotope, soil-water, water-table, trench-flow, tracer, and geochemistry data.</t>
+          <t>Reference IDs 169; 170; approach=E+M; tracer=Iso+Ions+EC+Dyes; flow=S+SS</t>
         </is>
       </c>
     </row>
@@ -6267,17 +6331,17 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Publication</t>
+          <t>Official_Repository</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Maimai database publication DOI</t>
+          <t>Maimai HydroShare repository</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1002/hyp.14112</t>
+          <t>https://www.hydroshare.org/resource/a292cb65a5d24a31a60978b2ab390266/</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -6292,29 +6356,29 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Data paper confirms Maimai M8 database is publicly available on HydroShare.</t>
+          <t>HydroShare repository contains public Maimai M8 rainfall-runoff, isotope, soil-water, water-table, trench-flow, tracer, and geochemistry data.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>WS10, H.J. Andrews, Oregon, United States</t>
+          <t>Maimai M8 experimental catchment, New Zealand</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Official_Repository</t>
+          <t>Publication</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Andrews LTER HF024</t>
+          <t>Maimai database publication DOI</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://andlter.forestry.oregonstate.edu/data/abstract.aspx?dbcode=HF024</t>
+          <t>https://doi.org/10.1002/hyp.14112</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -6329,14 +6393,14 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>HF024 provides downloadable WS10 isotope, chemistry, tracer, precipitation/streamflow, and soil-moisture data.</t>
+          <t>Data paper confirms Maimai M8 database is publicly available on HydroShare.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>WS10, H.J. Andrews, Oregon, United States</t>
+          <t>Maimai M8 experimental catchment, New Zealand</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -6346,34 +6410,34 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Andrews WS10 data index</t>
+          <t>Maimai HydroShare repository</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://andrewsforest.oregonstate.edu/sites/default/files/lter/data/weather/portal/GSWS10/data/index.html</t>
+          <t>https://www.hydroshare.org/resource/a292cb65a5d24a31a60978b2ab390266/</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Public Maimai M8 rainfall-runoff, isotope, groundwater and soil-water data</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>WS10 portal lists downloadable gaging station data and water-sample files.</t>
+          <t>HydroShare database contains public Maimai observations from multiple research phases.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>WS10, H.J. Andrews, Oregon, United States</t>
+          <t>Maimai M8 experimental catchment, New Zealand</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -6383,160 +6447,160 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Andrews LTER data list</t>
+          <t>CUAHSI HydroShare Maimai Experimental Watershed</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://andrewsforest.oregonstate.edu/data/data-all</t>
+          <t>https://www.hydroshare.org/resource/a292cb65a5d24a31a60978b2ab390266/</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Official/project repository public-data status and variable availability</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Data list documents public benchmark precipitation, streamflow, soil moisture, isotope, and chemistry packages.</t>
+          <t>Public Maimai HydroShare database includes rainfall-runoff, isotopes, soil-water/matric potential, water-table/well, trench-flow/tracer and geochemical data.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Athabasca Oil Sands region, Alberta, Canada</t>
+          <t>WS10, H.J. Andrews, Oregon, United States</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Official_Repository</t>
+          <t>McMillan</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Oil Sands Monitoring surface water quality</t>
+          <t>ProcessDatabase3-filtered.xlsx</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://osmdatacatalog.alberta.ca/dataset/surface-water-quality-discrete</t>
+          <t>https://doi.org/10.1016/j.jhydrol.2012.05.023</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Watershed metadata and Level-1 runoff process aggregation</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>OSM catalog provides downloadable surface-water quality data including stable isotopes and physical parameters.</t>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Athabasca Oil Sands region, Alberta, Canada</t>
+          <t>WS10, H.J. Andrews, Oregon, United States</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Official_Repository</t>
+          <t>Penna_Part2</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Canada Open Data groundwater quality</t>
+          <t>Penna_globalsynthesis_DB_Part2_update_2026_01.csv</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://open.canada.ca/data/en/dataset/9e2eebb1-d31a-4cc0-9434-fa5fe2c90684</t>
+          <t>https://doi.org/10.5281/zenodo.15123553</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Catchment fuzzy match and runoff-process labels</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Government dataset provides groundwater quality including EC and related parameters in the oil sands region.</t>
+          <t>Matched to Coweeta WS10; HJ Andrews Look Out; HJ Andrews Mack; HJ Andrews WS01; HJ Andrews WS02; HJ Andrews WS03; HJ Andrews WS08; HJ Andrews WS09 (+1 more) with process labels: (Perched) WT/GW dynamics and changes in GW storage; Dynamics of saturated areas; IEOF; Lateral flow; Lateral preferential flow; Macropore flow (no specifical vert/lat); Preferential flow (no specifica vert/lat); SEOF; Slow/deep SubFlow; SubFlow; Subsurface hillslope-stream connectivity; Water moveme</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Pedler Creek, Willunga Basin, Australia</t>
+          <t>WS10, H.J. Andrews, Oregon, United States</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Penna_Part1</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Pedler Creek GitHub repository</t>
+          <t>Penna_globalsynthesis_DB_Part1.csv</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/daniel-partington/Pedler_creek_streamflow_generation/tree/1.0</t>
+          <t>https://doi.org/10.5281/zenodo.15123553</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Reference-level approach/tracer/flow type</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Repository contains model input files for the HESS Pedler Creek streamflow-generation study.</t>
+          <t>Reference IDs 114; 117; 173; 174; 177; 202; 204; 238; 251; 257; approach=E; E+M; M; tracer=; flow=S; S+SS; SS</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Pedler Creek, Willunga Basin, Australia</t>
+          <t>WS10, H.J. Andrews, Oregon, United States</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Publication</t>
+          <t>Official_Repository</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Pedler Creek HESS relations page</t>
+          <t>Andrews LTER HF024</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://hess.copernicus.org/articles/25/4299/2021/hess-25-4299-2021-relations.html</t>
+          <t>https://andlter.forestry.oregonstate.edu/data/abstract.aspx?dbcode=HF024</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -6551,14 +6615,14 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>HESS page cites Zenodo/GitHub model inputs and SA Water Data Services Pedler Creek station.</t>
+          <t>HF024 provides downloadable WS10 isotope, chemistry, tracer, precipitation/streamflow, and soil-moisture data.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Pedler Creek, Willunga Basin, Australia</t>
+          <t>WS10, H.J. Andrews, Oregon, United States</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -6568,12 +6632,12 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Willunga Basin groundwater report</t>
+          <t>Andrews WS10 data index</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://www.waterconnect.sa.gov.au/Content/Publications/DEW/Willunga_Basin_GW_Resources_1998.pdf</t>
+          <t>https://andrewsforest.oregonstate.edu/sites/default/files/lter/data/weather/portal/GSWS10/data/index.html</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -6588,14 +6652,14 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Government report documents groundwater monitoring, salinity/EC, hydrochemistry, isotope recommendations, and Pedler Creek groundwater discharge.</t>
+          <t>WS10 portal lists downloadable gaging station data and water-sample files.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Conventwald Basin, Black Forest Mountains, Germany</t>
+          <t>WS10, H.J. Andrews, Oregon, United States</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -6605,12 +6669,12 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>GFZ Conventwald dataset</t>
+          <t>Andrews LTER data list</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://dataservices.gfz-potsdam.de/panmetaworks/showshort.php?id=39eae896-e323-11eb-9603-497c92695674</t>
+          <t>https://andrewsforest.oregonstate.edu/data/data-all</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -6625,103 +6689,103 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>GFZ dataset documents rainfall/throughfall, creek discharge, groundwater, subsurface flow, chemistry, and Mg/Li isotope observations.</t>
+          <t>Data list documents public benchmark precipitation, streamflow, soil moisture, isotope, and chemistry packages.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Conventwald Basin, Black Forest Mountains, Germany</t>
+          <t>WS10, H.J. Andrews, Oregon, United States</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Project_Website</t>
+          <t>Official_Repository</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>FVA Conventwald official page</t>
+          <t>Andrews Forest LTER / EDI</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://www.fva-bw.de/daten-tools/monitoring/oekosystemstudie-conventwald</t>
+          <t>https://andrewsforest.oregonstate.edu/data</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Official/project repository public-data status and variable availability</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Official FVA page describes long-term water and element-cycle monitoring at Conventwald.</t>
+          <t>Andrews LTER/EDI provides public precipitation, streamflow, soil moisture/temperature, isotope, chemistry and snow-related datasets.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Mt. Hermon Range, Israel, Syria, and Lebanon</t>
+          <t>Athabasca Oil Sands region, Alberta, Canada</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Publication</t>
+          <t>McMillan</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Mt. Hermon Scientific Reports article</t>
+          <t>ProcessDatabase3-filtered.xlsx</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41598-025-29454-9</t>
+          <t>https://doi.org/10.1016/j.ejrh.2015.12.062</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Watershed metadata and Level-1 runoff process aggregation</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Article describes limited spring discharge, groundwater/head, chemistry/solute observations and explicitly notes poor gauging and non-shared data.</t>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Mt. Hermon Range, Israel, Syria, and Lebanon</t>
+          <t>Athabasca Oil Sands region, Alberta, Canada</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Publication</t>
+          <t>Official_Repository</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Mt. Hermon groundwater modeling paper</t>
+          <t>Oil Sands Monitoring surface water quality</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://www.mdpi.com/2073-4441/7/7/3978</t>
+          <t>https://osmdatacatalog.alberta.ca/dataset/surface-water-quality-discrete</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -6736,14 +6800,14 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Paper documents limited groundwater data and modeling in the northeastern Mt. Hermon/Barada-Awaj area.</t>
+          <t>OSM catalog provides downloadable surface-water quality data including stable isotopes and physical parameters.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Freiberger Mulde, Germany</t>
+          <t>Athabasca Oil Sands region, Alberta, Canada</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -6753,12 +6817,12 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Saxon Flood Center Mulde discharge</t>
+          <t>Canada Open Data groundwater quality</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://www.hochwasserzentrum.sachsen.de/umwelt/infosysteme/lhwz/flussgebiet-mulde.html</t>
+          <t>https://open.canada.ca/data/en/dataset/9e2eebb1-d31a-4cc0-9434-fa5fe2c90684</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -6773,66 +6837,66 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Official portal provides annual discharge lists for Freiberger Mulde gauges.</t>
+          <t>Government dataset provides groundwater quality including EC and related parameters in the oil sands region.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Freiberger Mulde, Germany</t>
+          <t>Pedler Creek, Willunga Basin, Australia</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Official_Repository</t>
+          <t>McMillan</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>B2FIND eastern German isotope dataset</t>
+          <t>ProcessDatabase3-filtered.xlsx</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://b2find.eudat.eu/dataset/d78a5ff2-14ce-5ff8-b033-7d8a1d65f7da</t>
+          <t>https://doi.org/10.5194/hess-25-4299-2021</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Watershed metadata and Level-1 runoff process aggregation</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Dataset includes seasonal isotope and field water-chemistry measurements in Mulde/eastern German river systems.</t>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Freiberger Mulde, Germany</t>
+          <t>Pedler Creek, Willunga Basin, Australia</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Publication</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Freiberger Mulde water-quality article</t>
+          <t>Pedler Creek GitHub repository</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://link.springer.com/article/10.1007/s00767-022-00512-7</t>
+          <t>https://github.com/daniel-partington/Pedler_creek_streamflow_generation/tree/1.0</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -6847,29 +6911,29 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Article documents EC and water-quality sampling along the Freiberger Mulde.</t>
+          <t>Repository contains model input files for the HESS Pedler Creek streamflow-generation study.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Kostroma Catchment, Russia</t>
+          <t>Pedler Creek, Willunga Basin, Australia</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Publication</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Kostroma Hydrometeorological Center network</t>
+          <t>Pedler Creek HESS relations page</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://kostroma.meteorf.ru/o-czentre/nablyudatelnaya-set.html</t>
+          <t>https://hess.copernicus.org/articles/25/4299/2021/hess-25-4299-2021-relations.html</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -6884,29 +6948,29 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Regional service page documents meteorological, hydrological, and water-quality observation posts in Kostroma Oblast.</t>
+          <t>HESS page cites Zenodo/GitHub model inputs and SA Water Data Services Pedler Creek station.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Kostroma Catchment, Russia</t>
+          <t>Pedler Creek, Willunga Basin, Australia</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Publication</t>
+          <t>Official_Repository</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Upper Volga spring flood modeling DOI</t>
+          <t>Willunga Basin groundwater report</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.5194/adgeo-9-115-2006</t>
+          <t>https://www.waterconnect.sa.gov.au/Content/Publications/DEW/Willunga_Basin_GW_Resources_1998.pdf</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -6921,79 +6985,671 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Cited paper supports use of regional hydrometeorological/snowmelt-runoff information but no public watershed repository was found.</t>
+          <t>Government report documents groundwater monitoring, salinity/EC, hydrochemistry, isotope recommendations, and Pedler Creek groundwater discharge.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Point Peter Brook watershed, New York, United States</t>
+          <t>Conventwald Basin, Black Forest Mountains, Germany</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Publication</t>
+          <t>McMillan</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Point Peter Brook cited DOI</t>
+          <t>ProcessDatabase3-filtered.xlsx</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.jhydrol.2007.05.007</t>
+          <t>https://doi.org/10.1002/hyp.142</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Observation/public-data decision support</t>
+          <t>Watershed metadata and Level-1 runoff process aggregation</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Cited publication supports riparian/hillslope contributions to storm runoff at Point Peter Brook.</t>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
+          <t>Conventwald Basin, Black Forest Mountains, Germany</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Official_Repository</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>GFZ Conventwald dataset</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>https://dataservices.gfz-potsdam.de/panmetaworks/showshort.php?id=39eae896-e323-11eb-9603-497c92695674</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Observation/public-data decision support</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>GFZ dataset documents rainfall/throughfall, creek discharge, groundwater, subsurface flow, chemistry, and Mg/Li isotope observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Conventwald Basin, Black Forest Mountains, Germany</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Project_Website</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>FVA Conventwald official page</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fva-bw.de/daten-tools/monitoring/oekosystemstudie-conventwald</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Observation/public-data decision support</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Official FVA page describes long-term water and element-cycle monitoring at Conventwald.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Mt. Hermon Range, Israel, Syria, and Lebanon</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>McMillan</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>ProcessDatabase3-filtered.xlsx</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/wrcr.20229</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Mt. Hermon Range, Israel, Syria, and Lebanon</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Publication</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Mt. Hermon Scientific Reports article</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41598-025-29454-9</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>Observation/public-data decision support</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Article describes limited spring discharge, groundwater/head, chemistry/solute observations and explicitly notes poor gauging and non-shared data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Mt. Hermon Range, Israel, Syria, and Lebanon</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Publication</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Mt. Hermon groundwater modeling paper</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mdpi.com/2073-4441/7/7/3978</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Observation/public-data decision support</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Paper documents limited groundwater data and modeling in the northeastern Mt. Hermon/Barada-Awaj area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Mt. Hermon Range, Israel, Syria, and Lebanon</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Official_Repository</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Publication record / Mt. Hermon Aquifer studies</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41598-025-29454-9</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Official/project repository public-data status and variable availability</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Mt. Hermon publications document limited spring discharge, groundwater, chemistry/isotope and snowmelt recharge evidence, but no official open data portal was verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Freiberger Mulde, Germany</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>McMillan</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>ProcessDatabase3-filtered.xlsx</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s12665-016-5750-y</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Freiberger Mulde, Germany</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Official_Repository</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Saxon Flood Center Mulde discharge</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hochwasserzentrum.sachsen.de/umwelt/infosysteme/lhwz/flussgebiet-mulde.html</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Observation/public-data decision support</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Official portal provides annual discharge lists for Freiberger Mulde gauges.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Freiberger Mulde, Germany</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Official_Repository</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>B2FIND eastern German isotope dataset</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>https://b2find.eudat.eu/dataset/d78a5ff2-14ce-5ff8-b033-7d8a1d65f7da</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Observation/public-data decision support</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Dataset includes seasonal isotope and field water-chemistry measurements in Mulde/eastern German river systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Freiberger Mulde, Germany</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Publication</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Freiberger Mulde water-quality article</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/article/10.1007/s00767-022-00512-7</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Observation/public-data decision support</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Article documents EC and water-quality sampling along the Freiberger Mulde.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Freiberger Mulde, Germany</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Official_Repository</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Saxon State Flood Center / Mulde discharge</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hochwasserzentrum.sachsen.de/umwelt/infosysteme/lhwz/flussgebiet-mulde.html</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Official/project repository public-data status and variable availability</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Saxon Flood Center provides official discharge downloads; literature/B2FIND support isotope/EC observations, but headwater-study auxiliary data downloads were not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Kostroma Catchment, Russia</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>McMillan</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>ProcessDatabase3-filtered.xlsx</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5194/adgeo-9-115-2006</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Kostroma Catchment, Russia</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Kostroma Hydrometeorological Center network</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>https://kostroma.meteorf.ru/o-czentre/nablyudatelnaya-set.html</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>Observation/public-data decision support</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Regional service page documents meteorological, hydrological, and water-quality observation posts in Kostroma Oblast.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Kostroma Catchment, Russia</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Publication</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Upper Volga spring flood modeling DOI</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5194/adgeo-9-115-2006</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Observation/public-data decision support</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>Cited paper supports use of regional hydrometeorological/snowmelt-runoff information but no public watershed repository was found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
           <t>Point Peter Brook watershed, New York, United States</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>McMillan</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>ProcessDatabase3-filtered.xlsx</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jhydrol.2007.05.007</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Watershed metadata and Level-1 runoff process aggregation</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>Primary McMillan-derived row used for watershed metadata, citation and Level-1 runoff process flags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Point Peter Brook watershed, New York, United States</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
         <is>
           <t>Publication</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Point Peter Brook cited DOI</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jhydrol.2007.05.007</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>Observation/public-data decision support</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>Cited publication supports riparian/hillslope contributions to storm runoff at Point Peter Brook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Point Peter Brook watershed, New York, United States</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Publication</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
         <is>
           <t>Point Peter Brook sulfate publication</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D82" s="2" t="inlineStr">
         <is>
           <t>https://link.springer.com/article/10.1007/s10661-007-9830-z</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E82" s="2" t="inlineStr">
         <is>
           <t>2026-06-02</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F82" s="2" t="inlineStr">
         <is>
           <t>Observation/public-data decision support</t>
         </is>
       </c>
-      <c r="G66" s="2" t="inlineStr">
+      <c r="G82" s="2" t="inlineStr">
         <is>
           <t>Publication abstract documents rainfall/throughfall, groundwater, stream/storm chemistry, sulfate, isotopic methods, and wetland/riparian comparisons.</t>
         </is>

</xml_diff>